<commit_message>
Actualización de datos 12/10/2026
</commit_message>
<xml_diff>
--- a/data/semestral.xlsx
+++ b/data/semestral.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsilvestre\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D3DD91-D8FB-4F6F-ABF9-86D8ECFB25BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12840" yWindow="792" windowWidth="10980" windowHeight="12216" firstSheet="2" activeTab="2"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RACIONES DE COMEDORES ABRIL " sheetId="1" r:id="rId1"/>
@@ -22,7 +28,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'RACIONES DE COMEDORES ABRIL '!$A$1:$O$133</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'RACIONES DE COMEDORES ABRIL '!$1:$6</definedName>
   </definedNames>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,12 +44,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="248">
   <si>
     <t>MODALIDAD</t>
   </si>
@@ -782,11 +791,17 @@
   <si>
     <t>261, 494</t>
   </si>
+  <si>
+    <t>julio</t>
+  </si>
+  <si>
+    <t>La Loma</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="7">
     <numFmt numFmtId="44" formatCode="_-&quot;Q&quot;* #,##0.00_-;\-&quot;Q&quot;* #,##0.00_-;_-&quot;Q&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
@@ -794,7 +809,7 @@
     <numFmt numFmtId="165" formatCode="_-&quot;Q&quot;* #,##0.00_-;\-&quot;Q&quot;* #,##0.00_-;_-&quot;Q&quot;* &quot;-&quot;??_-;_-@"/>
     <numFmt numFmtId="166" formatCode="#,##0_);\(#,##0\)"/>
     <numFmt numFmtId="167" formatCode="#,##0_ ;\-#,##0\ "/>
-    <numFmt numFmtId="169" formatCode="0.0000%"/>
+    <numFmt numFmtId="168" formatCode="0.0000%"/>
   </numFmts>
   <fonts count="21" x14ac:knownFonts="1">
     <font>
@@ -1043,7 +1058,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -1330,19 +1345,6 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -1350,88 +1352,11 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1444,80 +1369,7 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1527,7 +1379,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="295">
+  <cellXfs count="285">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2161,41 +2013,43 @@
     <xf numFmtId="44" fontId="11" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="9" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="9" fillId="15" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="9" fillId="15" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="9" fillId="15" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="9" fillId="15" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="9" fillId="15" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="9" fillId="15" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2269,42 +2123,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="9" fillId="15" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="9" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="9" fillId="15" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="3" builtinId="3"/>
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -2344,9 +2174,9 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-GT"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2383,7 +2213,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2430,7 +2259,7 @@
                 <a:noFill/>
               </a:ln>
             </c:spPr>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000001-0F28-4C88-992A-66142F6CB08B}"/>
               </c:ext>
@@ -2447,7 +2276,7 @@
                 <a:noFill/>
               </a:ln>
             </c:spPr>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000003-0F28-4C88-992A-66142F6CB08B}"/>
               </c:ext>
@@ -2464,7 +2293,7 @@
                 <a:noFill/>
               </a:ln>
             </c:spPr>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000005-0F28-4C88-992A-66142F6CB08B}"/>
               </c:ext>
@@ -2473,7 +2302,6 @@
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
-              <c:layout/>
               <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
@@ -2497,7 +2325,8 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
-              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-0F28-4C88-992A-66142F6CB08B}"/>
                 </c:ext>
@@ -2505,7 +2334,6 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
-              <c:layout/>
               <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
@@ -2529,7 +2357,8 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
-              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-0F28-4C88-992A-66142F6CB08B}"/>
                 </c:ext>
@@ -2537,7 +2366,6 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="2"/>
-              <c:layout/>
               <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
@@ -2561,7 +2389,8 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
-              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000005-0F28-4C88-992A-66142F6CB08B}"/>
                 </c:ext>
@@ -2598,7 +2427,7 @@
             <c:showBubbleSize val="1"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
             </c:extLst>
           </c:dLbls>
@@ -2623,7 +2452,7 @@
             <c:numRef>
               <c:f>'[2]GRAFICA '!$B$57:$B$59</c:f>
               <c:numCache>
-                <c:formatCode>#,##0_ ;\-#,##0\ </c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>184274</c:v>
@@ -2637,7 +2466,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-0F28-4C88-992A-66142F6CB08B}"/>
             </c:ext>
@@ -2663,7 +2492,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2711,9 +2539,9 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-GT"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2750,7 +2578,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2797,7 +2624,7 @@
                 <a:noFill/>
               </a:ln>
             </c:spPr>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000001-58B8-4A87-A027-FEFF73D4BF12}"/>
               </c:ext>
@@ -2814,7 +2641,7 @@
                 <a:noFill/>
               </a:ln>
             </c:spPr>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000003-58B8-4A87-A027-FEFF73D4BF12}"/>
               </c:ext>
@@ -2865,7 +2692,10 @@
               <c:showSerName val="1"/>
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
-              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:showDataLabelsRange val="0"/>
+                </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-58B8-4A87-A027-FEFF73D4BF12}"/>
                 </c:ext>
@@ -2915,7 +2745,10 @@
               <c:showSerName val="1"/>
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
-              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:showDataLabelsRange val="0"/>
+                </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-58B8-4A87-A027-FEFF73D4BF12}"/>
                 </c:ext>
@@ -2952,7 +2785,7 @@
             <c:showBubbleSize val="1"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
             </c:extLst>
           </c:dLbls>
@@ -2974,7 +2807,7 @@
             <c:numRef>
               <c:f>'[2]GRAFICA '!$B$63:$B$64</c:f>
               <c:numCache>
-                <c:formatCode>#,##0_ ;\-#,##0\ </c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>4222963</c:v>
@@ -2985,7 +2818,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-58B8-4A87-A027-FEFF73D4BF12}"/>
             </c:ext>
@@ -3011,7 +2844,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3059,9 +2891,9 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-GT"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3097,7 +2929,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -3116,7 +2947,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>NO. RACIONES PROYECTADAS</c:v>
+                  <c:v> NO. RACIONES PROYECTADAS </c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3132,9 +2963,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'GRAFICA '!$A$7:$B$24</c:f>
+              <c:f>'GRAFICA '!$A$7:$B$26</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="18"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>Enero</c:v>
@@ -3155,39 +2986,45 @@
                     <c:v>junio </c:v>
                   </c:pt>
                   <c:pt idx="6">
+                    <c:v>julio</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
                     <c:v>Enero</c:v>
                   </c:pt>
-                  <c:pt idx="7">
+                  <c:pt idx="8">
                     <c:v>Febrero</c:v>
                   </c:pt>
-                  <c:pt idx="8">
+                  <c:pt idx="9">
                     <c:v>Marzo</c:v>
                   </c:pt>
-                  <c:pt idx="9">
+                  <c:pt idx="10">
                     <c:v>abril </c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="11">
                     <c:v>mayo </c:v>
                   </c:pt>
-                  <c:pt idx="11">
+                  <c:pt idx="12">
                     <c:v>junio </c:v>
                   </c:pt>
-                  <c:pt idx="12">
+                  <c:pt idx="13">
+                    <c:v>julio</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
                     <c:v>Enero</c:v>
                   </c:pt>
-                  <c:pt idx="13">
+                  <c:pt idx="15">
                     <c:v>Febrero</c:v>
                   </c:pt>
-                  <c:pt idx="14">
+                  <c:pt idx="16">
                     <c:v>Marzo</c:v>
                   </c:pt>
-                  <c:pt idx="15">
+                  <c:pt idx="17">
                     <c:v>abril </c:v>
                   </c:pt>
-                  <c:pt idx="16">
+                  <c:pt idx="18">
                     <c:v>mayo </c:v>
                   </c:pt>
-                  <c:pt idx="17">
+                  <c:pt idx="19">
                     <c:v>junio </c:v>
                   </c:pt>
                 </c:lvl>
@@ -3195,10 +3032,10 @@
                   <c:pt idx="0">
                     <c:v>Banquetes de Guatemala </c:v>
                   </c:pt>
-                  <c:pt idx="6">
+                  <c:pt idx="7">
                     <c:v>Tecno Suministros </c:v>
                   </c:pt>
-                  <c:pt idx="12">
+                  <c:pt idx="14">
                     <c:v>El Rosario</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3207,10 +3044,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'GRAFICA '!$C$7:$C$24</c:f>
+              <c:f>'GRAFICA '!$C$7:$C$26</c:f>
               <c:numCache>
                 <c:formatCode>#,##0_ ;\-#,##0\ </c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="20"/>
                 <c:pt idx="0">
                   <c:v>484110</c:v>
                 </c:pt>
@@ -3230,45 +3067,51 @@
                   <c:v>617040</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>768125</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>129240</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>133412</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>152560</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>133725</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>139600</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>146080</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="13">
+                  <c:v>219190</c:v>
+                </c:pt>
+                <c:pt idx="14">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>109100</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>125510</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>108395</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>114100</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>119805</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-E236-46D0-B095-2510CA023FC3}"/>
             </c:ext>
@@ -3283,7 +3126,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>NO. DE RACIONES PAGADAS</c:v>
+                  <c:v> NO. DE RACIONES PAGADAS </c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3299,9 +3142,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'GRAFICA '!$A$7:$B$24</c:f>
+              <c:f>'GRAFICA '!$A$7:$B$26</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="18"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>Enero</c:v>
@@ -3322,39 +3165,45 @@
                     <c:v>junio </c:v>
                   </c:pt>
                   <c:pt idx="6">
+                    <c:v>julio</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
                     <c:v>Enero</c:v>
                   </c:pt>
-                  <c:pt idx="7">
+                  <c:pt idx="8">
                     <c:v>Febrero</c:v>
                   </c:pt>
-                  <c:pt idx="8">
+                  <c:pt idx="9">
                     <c:v>Marzo</c:v>
                   </c:pt>
-                  <c:pt idx="9">
+                  <c:pt idx="10">
                     <c:v>abril </c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="11">
                     <c:v>mayo </c:v>
                   </c:pt>
-                  <c:pt idx="11">
+                  <c:pt idx="12">
                     <c:v>junio </c:v>
                   </c:pt>
-                  <c:pt idx="12">
+                  <c:pt idx="13">
+                    <c:v>julio</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
                     <c:v>Enero</c:v>
                   </c:pt>
-                  <c:pt idx="13">
+                  <c:pt idx="15">
                     <c:v>Febrero</c:v>
                   </c:pt>
-                  <c:pt idx="14">
+                  <c:pt idx="16">
                     <c:v>Marzo</c:v>
                   </c:pt>
-                  <c:pt idx="15">
+                  <c:pt idx="17">
                     <c:v>abril </c:v>
                   </c:pt>
-                  <c:pt idx="16">
+                  <c:pt idx="18">
                     <c:v>mayo </c:v>
                   </c:pt>
-                  <c:pt idx="17">
+                  <c:pt idx="19">
                     <c:v>junio </c:v>
                   </c:pt>
                 </c:lvl>
@@ -3362,10 +3211,10 @@
                   <c:pt idx="0">
                     <c:v>Banquetes de Guatemala </c:v>
                   </c:pt>
-                  <c:pt idx="6">
+                  <c:pt idx="7">
                     <c:v>Tecno Suministros </c:v>
                   </c:pt>
-                  <c:pt idx="12">
+                  <c:pt idx="14">
                     <c:v>El Rosario</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3374,10 +3223,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'GRAFICA '!$D$7:$D$24</c:f>
+              <c:f>'GRAFICA '!$D$7:$D$26</c:f>
               <c:numCache>
                 <c:formatCode>#,##0_ ;\-#,##0\ </c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="20"/>
                 <c:pt idx="0">
                   <c:v>484033</c:v>
                 </c:pt>
@@ -3397,45 +3246,51 @@
                   <c:v>564625</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>736664</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>120858</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>131583</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>150810</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>133684</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>136960</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>145437</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="13">
+                  <c:v>219190</c:v>
+                </c:pt>
+                <c:pt idx="14">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="15">
                   <c:v>101841</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>103404</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>94818</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>104314</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>110598</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-E236-46D0-B095-2510CA023FC3}"/>
             </c:ext>
@@ -3450,7 +3305,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>NO. DE RACIONES NO PAGADAS </c:v>
+                  <c:v> NO. DE RACIONES NO PAGADAS  </c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3463,9 +3318,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'GRAFICA '!$A$7:$B$24</c:f>
+              <c:f>'GRAFICA '!$A$7:$B$26</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="18"/>
+                <c:ptCount val="20"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>Enero</c:v>
@@ -3486,39 +3341,45 @@
                     <c:v>junio </c:v>
                   </c:pt>
                   <c:pt idx="6">
+                    <c:v>julio</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
                     <c:v>Enero</c:v>
                   </c:pt>
-                  <c:pt idx="7">
+                  <c:pt idx="8">
                     <c:v>Febrero</c:v>
                   </c:pt>
-                  <c:pt idx="8">
+                  <c:pt idx="9">
                     <c:v>Marzo</c:v>
                   </c:pt>
-                  <c:pt idx="9">
+                  <c:pt idx="10">
                     <c:v>abril </c:v>
                   </c:pt>
-                  <c:pt idx="10">
+                  <c:pt idx="11">
                     <c:v>mayo </c:v>
                   </c:pt>
-                  <c:pt idx="11">
+                  <c:pt idx="12">
                     <c:v>junio </c:v>
                   </c:pt>
-                  <c:pt idx="12">
+                  <c:pt idx="13">
+                    <c:v>julio</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
                     <c:v>Enero</c:v>
                   </c:pt>
-                  <c:pt idx="13">
+                  <c:pt idx="15">
                     <c:v>Febrero</c:v>
                   </c:pt>
-                  <c:pt idx="14">
+                  <c:pt idx="16">
                     <c:v>Marzo</c:v>
                   </c:pt>
-                  <c:pt idx="15">
+                  <c:pt idx="17">
                     <c:v>abril </c:v>
                   </c:pt>
-                  <c:pt idx="16">
+                  <c:pt idx="18">
                     <c:v>mayo </c:v>
                   </c:pt>
-                  <c:pt idx="17">
+                  <c:pt idx="19">
                     <c:v>junio </c:v>
                   </c:pt>
                 </c:lvl>
@@ -3526,10 +3387,10 @@
                   <c:pt idx="0">
                     <c:v>Banquetes de Guatemala </c:v>
                   </c:pt>
-                  <c:pt idx="6">
+                  <c:pt idx="7">
                     <c:v>Tecno Suministros </c:v>
                   </c:pt>
-                  <c:pt idx="12">
+                  <c:pt idx="14">
                     <c:v>El Rosario</c:v>
                   </c:pt>
                 </c:lvl>
@@ -3538,10 +3399,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'GRAFICA '!$E$7:$E$24</c:f>
+              <c:f>'GRAFICA '!$E$7:$E$26</c:f>
               <c:numCache>
                 <c:formatCode>#,##0_ ;\-#,##0\ </c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="20"/>
                 <c:pt idx="0">
                   <c:v>77</c:v>
                 </c:pt>
@@ -3561,45 +3422,51 @@
                   <c:v>52415</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>31461</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>8382</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>1829</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>1750</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>41</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>2640</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>643</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="13">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>7259</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>22106</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>13577</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>9786</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
                   <c:v>9207</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-E236-46D0-B095-2510CA023FC3}"/>
             </c:ext>
@@ -3685,7 +3552,7 @@
         <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{31B77592-3AA2-468B-8A88-AE89B5EC5058}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3732,7 +3599,13 @@
     <xdr:ext cx="1790700" cy="628650"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="2" name="image2.png" title="Imagen">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3764,7 +3637,13 @@
     <xdr:ext cx="1009650" cy="457200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="image1.png"/>
+        <xdr:cNvPr id="3" name="image1.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3796,7 +3675,13 @@
     <xdr:ext cx="1009650" cy="457200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="image1.png"/>
+        <xdr:cNvPr id="4" name="image1.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3841,7 +3726,7 @@
         <xdr:cNvPr id="2" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0200-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3879,7 +3764,7 @@
         <xdr:cNvPr id="3" name="Chart 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0200-000006000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3914,7 +3799,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="3 Gráfico"/>
+        <xdr:cNvPr id="4" name="3 Gráfico">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -3935,7 +3826,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="EJECUCIÓN QUINCENA MAYO"/>
@@ -4583,7 +4474,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="RACIONES DE COMEDORES ABRIL "/>
@@ -4693,7 +4584,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -4745,7 +4636,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -4939,14 +4830,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A2:Q149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
@@ -5016,20 +4907,20 @@
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="7"/>
-      <c r="G5" s="255" t="s">
+      <c r="G5" s="257" t="s">
         <v>139</v>
       </c>
-      <c r="H5" s="255"/>
-      <c r="I5" s="253" t="s">
+      <c r="H5" s="257"/>
+      <c r="I5" s="255" t="s">
         <v>141</v>
       </c>
-      <c r="J5" s="253"/>
-      <c r="K5" s="253"/>
-      <c r="L5" s="253" t="s">
+      <c r="J5" s="255"/>
+      <c r="K5" s="255"/>
+      <c r="L5" s="255" t="s">
         <v>142</v>
       </c>
-      <c r="M5" s="253"/>
-      <c r="N5" s="253"/>
+      <c r="M5" s="255"/>
+      <c r="N5" s="255"/>
     </row>
     <row r="6" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
@@ -11605,16 +11496,16 @@
       <c r="O130" s="66"/>
     </row>
     <row r="131" spans="1:15" s="12" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="254" t="s">
+      <c r="A131" s="256" t="s">
         <v>143</v>
       </c>
-      <c r="B131" s="254"/>
-      <c r="C131" s="254"/>
-      <c r="D131" s="254"/>
-      <c r="E131" s="254"/>
-      <c r="F131" s="254"/>
-      <c r="G131" s="254"/>
-      <c r="H131" s="254"/>
+      <c r="B131" s="256"/>
+      <c r="C131" s="256"/>
+      <c r="D131" s="256"/>
+      <c r="E131" s="256"/>
+      <c r="F131" s="256"/>
+      <c r="G131" s="256"/>
+      <c r="H131" s="256"/>
       <c r="I131" s="14" t="e">
         <f>SUM(I7:I130)</f>
         <v>#REF!</v>
@@ -11666,7 +11557,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:Q131">
+  <autoFilter ref="A6:Q131" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="2">
       <colorFilter dxfId="1"/>
     </filterColumn>
@@ -11684,7 +11575,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:AQ1001"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -11763,32 +11654,32 @@
       <c r="AH1" s="75"/>
     </row>
     <row r="2" spans="1:42" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="271" t="s">
+      <c r="A2" s="273" t="s">
         <v>213</v>
       </c>
-      <c r="B2" s="272"/>
-      <c r="C2" s="272"/>
-      <c r="D2" s="272"/>
-      <c r="E2" s="272"/>
-      <c r="F2" s="272"/>
-      <c r="G2" s="272"/>
-      <c r="H2" s="272"/>
-      <c r="I2" s="272"/>
-      <c r="J2" s="272"/>
-      <c r="K2" s="272"/>
-      <c r="L2" s="272"/>
-      <c r="M2" s="272"/>
-      <c r="N2" s="272"/>
-      <c r="O2" s="272"/>
-      <c r="P2" s="272"/>
-      <c r="Q2" s="272"/>
-      <c r="R2" s="272"/>
-      <c r="S2" s="272"/>
-      <c r="T2" s="272"/>
-      <c r="U2" s="272"/>
-      <c r="V2" s="272"/>
-      <c r="W2" s="272"/>
-      <c r="X2" s="272"/>
+      <c r="B2" s="274"/>
+      <c r="C2" s="274"/>
+      <c r="D2" s="274"/>
+      <c r="E2" s="274"/>
+      <c r="F2" s="274"/>
+      <c r="G2" s="274"/>
+      <c r="H2" s="274"/>
+      <c r="I2" s="274"/>
+      <c r="J2" s="274"/>
+      <c r="K2" s="274"/>
+      <c r="L2" s="274"/>
+      <c r="M2" s="274"/>
+      <c r="N2" s="274"/>
+      <c r="O2" s="274"/>
+      <c r="P2" s="274"/>
+      <c r="Q2" s="274"/>
+      <c r="R2" s="274"/>
+      <c r="S2" s="274"/>
+      <c r="T2" s="274"/>
+      <c r="U2" s="274"/>
+      <c r="V2" s="274"/>
+      <c r="W2" s="274"/>
+      <c r="X2" s="274"/>
       <c r="Y2" s="75"/>
       <c r="Z2" s="75"/>
       <c r="AA2" s="75"/>
@@ -11995,108 +11886,108 @@
       <c r="H8" s="84"/>
       <c r="I8" s="84"/>
       <c r="J8" s="84"/>
-      <c r="K8" s="266" t="s">
+      <c r="K8" s="268" t="s">
         <v>216</v>
       </c>
-      <c r="L8" s="267"/>
-      <c r="M8" s="267"/>
-      <c r="N8" s="267"/>
-      <c r="O8" s="267"/>
-      <c r="P8" s="268"/>
-      <c r="Q8" s="266" t="s">
+      <c r="L8" s="269"/>
+      <c r="M8" s="269"/>
+      <c r="N8" s="269"/>
+      <c r="O8" s="269"/>
+      <c r="P8" s="270"/>
+      <c r="Q8" s="268" t="s">
         <v>217</v>
       </c>
-      <c r="R8" s="267"/>
-      <c r="S8" s="267"/>
-      <c r="T8" s="267"/>
-      <c r="U8" s="267"/>
-      <c r="V8" s="268"/>
-      <c r="W8" s="266" t="s">
+      <c r="R8" s="269"/>
+      <c r="S8" s="269"/>
+      <c r="T8" s="269"/>
+      <c r="U8" s="269"/>
+      <c r="V8" s="270"/>
+      <c r="W8" s="268" t="s">
         <v>167</v>
       </c>
-      <c r="X8" s="269"/>
-      <c r="Y8" s="269"/>
-      <c r="Z8" s="269"/>
-      <c r="AA8" s="269"/>
-      <c r="AB8" s="270"/>
-      <c r="AC8" s="266" t="s">
+      <c r="X8" s="271"/>
+      <c r="Y8" s="271"/>
+      <c r="Z8" s="271"/>
+      <c r="AA8" s="271"/>
+      <c r="AB8" s="272"/>
+      <c r="AC8" s="268" t="s">
         <v>218</v>
       </c>
-      <c r="AD8" s="267"/>
-      <c r="AE8" s="267"/>
-      <c r="AF8" s="267"/>
-      <c r="AG8" s="267"/>
-      <c r="AH8" s="267"/>
-      <c r="AI8" s="273" t="s">
+      <c r="AD8" s="269"/>
+      <c r="AE8" s="269"/>
+      <c r="AF8" s="269"/>
+      <c r="AG8" s="269"/>
+      <c r="AH8" s="269"/>
+      <c r="AI8" s="275" t="s">
         <v>219</v>
       </c>
-      <c r="AJ8" s="274"/>
-      <c r="AK8" s="274"/>
-      <c r="AL8" s="274"/>
-      <c r="AM8" s="274"/>
-      <c r="AN8" s="275"/>
+      <c r="AJ8" s="276"/>
+      <c r="AK8" s="276"/>
+      <c r="AL8" s="276"/>
+      <c r="AM8" s="276"/>
+      <c r="AN8" s="277"/>
     </row>
     <row r="9" spans="1:42" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="84"/>
       <c r="B9" s="85"/>
       <c r="C9" s="86"/>
       <c r="D9" s="84"/>
-      <c r="E9" s="279" t="s">
+      <c r="E9" s="281" t="s">
         <v>220</v>
       </c>
-      <c r="F9" s="280"/>
-      <c r="G9" s="279" t="s">
+      <c r="F9" s="282"/>
+      <c r="G9" s="281" t="s">
         <v>139</v>
       </c>
-      <c r="H9" s="280"/>
+      <c r="H9" s="282"/>
       <c r="I9" s="87"/>
       <c r="J9" s="87"/>
-      <c r="K9" s="266" t="s">
+      <c r="K9" s="268" t="s">
         <v>141</v>
       </c>
-      <c r="L9" s="267"/>
-      <c r="M9" s="268"/>
-      <c r="N9" s="266" t="s">
+      <c r="L9" s="269"/>
+      <c r="M9" s="270"/>
+      <c r="N9" s="268" t="s">
         <v>221</v>
       </c>
-      <c r="O9" s="267"/>
-      <c r="P9" s="268"/>
-      <c r="Q9" s="266" t="s">
+      <c r="O9" s="269"/>
+      <c r="P9" s="270"/>
+      <c r="Q9" s="268" t="s">
         <v>168</v>
       </c>
-      <c r="R9" s="267"/>
-      <c r="S9" s="268"/>
-      <c r="T9" s="266" t="s">
+      <c r="R9" s="269"/>
+      <c r="S9" s="270"/>
+      <c r="T9" s="268" t="s">
         <v>169</v>
       </c>
-      <c r="U9" s="267"/>
-      <c r="V9" s="268"/>
-      <c r="W9" s="266" t="s">
+      <c r="U9" s="269"/>
+      <c r="V9" s="270"/>
+      <c r="W9" s="268" t="s">
         <v>170</v>
       </c>
-      <c r="X9" s="269"/>
-      <c r="Y9" s="270"/>
-      <c r="Z9" s="266" t="s">
+      <c r="X9" s="271"/>
+      <c r="Y9" s="272"/>
+      <c r="Z9" s="268" t="s">
         <v>171</v>
       </c>
-      <c r="AA9" s="269"/>
-      <c r="AB9" s="270"/>
-      <c r="AC9" s="266" t="s">
+      <c r="AA9" s="271"/>
+      <c r="AB9" s="272"/>
+      <c r="AC9" s="268" t="s">
         <v>222</v>
       </c>
-      <c r="AD9" s="267"/>
-      <c r="AE9" s="268"/>
-      <c r="AF9" s="266" t="s">
+      <c r="AD9" s="269"/>
+      <c r="AE9" s="270"/>
+      <c r="AF9" s="268" t="s">
         <v>171</v>
       </c>
-      <c r="AG9" s="267"/>
-      <c r="AH9" s="267"/>
-      <c r="AI9" s="276"/>
-      <c r="AJ9" s="277"/>
-      <c r="AK9" s="277"/>
-      <c r="AL9" s="277"/>
-      <c r="AM9" s="277"/>
-      <c r="AN9" s="278"/>
+      <c r="AG9" s="269"/>
+      <c r="AH9" s="269"/>
+      <c r="AI9" s="278"/>
+      <c r="AJ9" s="279"/>
+      <c r="AK9" s="279"/>
+      <c r="AL9" s="279"/>
+      <c r="AM9" s="279"/>
+      <c r="AN9" s="280"/>
     </row>
     <row r="10" spans="1:42" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="109" t="s">
@@ -26722,7 +26613,7 @@
         <v>121500</v>
       </c>
     </row>
-    <row r="108" spans="1:42" s="104" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:42" s="104" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="135" t="e">
         <f t="shared" si="25"/>
         <v>#REF!</v>
@@ -26872,7 +26763,7 @@
         <v>162000</v>
       </c>
     </row>
-    <row r="109" spans="1:42" s="104" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:42" s="104" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="135" t="e">
         <f t="shared" si="25"/>
         <v>#REF!</v>
@@ -28817,23 +28708,23 @@
       </c>
     </row>
     <row r="122" spans="1:42" s="156" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="256" t="e">
+      <c r="A122" s="258" t="e">
         <f>+A121+1</f>
         <v>#REF!</v>
       </c>
-      <c r="B122" s="258" t="s">
+      <c r="B122" s="260" t="s">
         <v>15</v>
       </c>
-      <c r="C122" s="260" t="s">
+      <c r="C122" s="262" t="s">
         <v>208</v>
       </c>
-      <c r="D122" s="262" t="s">
+      <c r="D122" s="264" t="s">
         <v>1</v>
       </c>
-      <c r="E122" s="264">
+      <c r="E122" s="266">
         <v>100</v>
       </c>
-      <c r="F122" s="264">
+      <c r="F122" s="266">
         <v>150</v>
       </c>
       <c r="G122" s="150">
@@ -28967,12 +28858,12 @@
       </c>
     </row>
     <row r="123" spans="1:42" s="156" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="257"/>
-      <c r="B123" s="259"/>
-      <c r="C123" s="261"/>
-      <c r="D123" s="263"/>
-      <c r="E123" s="265"/>
-      <c r="F123" s="265"/>
+      <c r="A123" s="259"/>
+      <c r="B123" s="261"/>
+      <c r="C123" s="263"/>
+      <c r="D123" s="265"/>
+      <c r="E123" s="267"/>
+      <c r="F123" s="267"/>
       <c r="G123" s="150">
         <v>23</v>
       </c>
@@ -69185,7 +69076,7 @@
       <c r="AP1001" s="79"/>
     </row>
   </sheetData>
-  <autoFilter ref="A10:AQ137">
+  <autoFilter ref="A10:AQ137" xr:uid="{00000000-0009-0000-0000-000001000000}">
     <filterColumn colId="2">
       <colorFilter dxfId="0"/>
     </filterColumn>
@@ -69220,15 +69111,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A5:I69"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A5:I76"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" customWidth="1"/>
-    <col min="3" max="3" width="24" style="240" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" style="240" customWidth="1"/>
-    <col min="5" max="5" width="19.5546875" style="240" customWidth="1"/>
+    <col min="3" max="3" width="24" style="239" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" style="239" customWidth="1"/>
+    <col min="5" max="5" width="19.5546875" style="239" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" customWidth="1"/>
     <col min="7" max="7" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" bestFit="1" customWidth="1"/>
@@ -69238,844 +69129,995 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="243" t="s">
+    <row r="6" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="246" t="s">
         <v>159</v>
       </c>
-      <c r="B6" s="244" t="s">
+      <c r="B6" s="247" t="s">
         <v>160</v>
       </c>
-      <c r="C6" s="245" t="s">
+      <c r="C6" s="248" t="s">
         <v>236</v>
       </c>
-      <c r="D6" s="245" t="s">
+      <c r="D6" s="248" t="s">
         <v>237</v>
       </c>
-      <c r="E6" s="246" t="s">
+      <c r="E6" s="254" t="s">
         <v>238</v>
       </c>
-      <c r="H6" s="288" t="s">
+      <c r="H6" s="242" t="s">
         <v>240</v>
       </c>
-      <c r="I6" s="288" t="s">
+      <c r="I6" s="242" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="281" t="s">
+      <c r="A7" s="284" t="s">
         <v>161</v>
       </c>
-      <c r="B7" s="241" t="s">
+      <c r="B7" s="251" t="s">
         <v>233</v>
       </c>
-      <c r="C7" s="247">
+      <c r="C7" s="240">
         <v>484110</v>
       </c>
-      <c r="D7" s="247">
-        <f>390370+93663</f>
+      <c r="D7" s="240">
         <v>484033</v>
       </c>
-      <c r="E7" s="248">
-        <f t="shared" ref="E7:E9" si="0">C7-D7</f>
+      <c r="E7" s="252">
+        <f t="shared" ref="E7:E28" si="0">C7-D7</f>
         <v>77</v>
       </c>
-      <c r="H7" s="287" t="s">
+      <c r="H7" s="241" t="s">
         <v>161</v>
       </c>
-      <c r="I7" s="289">
+      <c r="I7" s="243">
         <v>184274</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="282"/>
-      <c r="B8" s="239" t="s">
+      <c r="A8" s="284"/>
+      <c r="B8" s="251" t="s">
         <v>234</v>
       </c>
-      <c r="C8" s="249">
+      <c r="C8" s="240">
         <v>442800</v>
       </c>
-      <c r="D8" s="249">
+      <c r="D8" s="240">
         <v>426896</v>
       </c>
-      <c r="E8" s="248">
+      <c r="E8" s="252">
         <f t="shared" si="0"/>
         <v>15904</v>
       </c>
-      <c r="H8" s="287" t="s">
+      <c r="H8" s="241" t="s">
         <v>164</v>
       </c>
-      <c r="I8" s="289">
+      <c r="I8" s="243">
         <v>15285</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="282"/>
-      <c r="B9" s="239" t="s">
+      <c r="A9" s="284"/>
+      <c r="B9" s="251" t="s">
         <v>235</v>
       </c>
-      <c r="C9" s="249">
+      <c r="C9" s="240">
         <v>513380</v>
       </c>
-      <c r="D9" s="249">
+      <c r="D9" s="240">
         <v>486936</v>
       </c>
-      <c r="E9" s="248">
+      <c r="E9" s="252">
         <f t="shared" si="0"/>
         <v>26444</v>
       </c>
-      <c r="H9" s="287" t="s">
+      <c r="H9" s="241" t="s">
         <v>166</v>
       </c>
-      <c r="I9" s="289">
+      <c r="I9" s="243">
         <v>61935</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="282"/>
-      <c r="B10" s="239" t="s">
+      <c r="A10" s="284"/>
+      <c r="B10" s="251" t="s">
         <v>165</v>
       </c>
-      <c r="C10" s="249">
+      <c r="C10" s="240">
         <v>490800</v>
       </c>
-      <c r="D10" s="249">
+      <c r="D10" s="240">
         <v>441840</v>
       </c>
-      <c r="E10" s="248">
-        <f>C10-D10</f>
+      <c r="E10" s="252">
+        <f t="shared" si="0"/>
         <v>48960</v>
       </c>
-      <c r="H10" s="287" t="s">
+      <c r="H10" s="241" t="s">
         <v>140</v>
       </c>
-      <c r="I10" s="287" t="s">
+      <c r="I10" s="241" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="282"/>
-      <c r="B11" s="239" t="s">
+      <c r="A11" s="284"/>
+      <c r="B11" s="251" t="s">
         <v>162</v>
       </c>
-      <c r="C11" s="249">
+      <c r="C11" s="240">
         <v>524800</v>
       </c>
-      <c r="D11" s="249">
+      <c r="D11" s="240">
         <v>484326</v>
       </c>
-      <c r="E11" s="248">
-        <f t="shared" ref="E11:E24" si="1">C11-D11</f>
+      <c r="E11" s="252">
+        <f t="shared" si="0"/>
         <v>40474</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="283"/>
-      <c r="B12" s="242" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="284"/>
+      <c r="B12" s="251" t="s">
         <v>163</v>
       </c>
-      <c r="C12" s="250">
+      <c r="C12" s="240">
         <v>617040</v>
       </c>
-      <c r="D12" s="250">
+      <c r="D12" s="240">
         <v>564625</v>
       </c>
-      <c r="E12" s="251">
+      <c r="E12" s="252">
+        <f t="shared" si="0"/>
+        <v>52415</v>
+      </c>
+      <c r="H12" s="242" t="s">
+        <v>243</v>
+      </c>
+      <c r="I12" s="242" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="284"/>
+      <c r="B13" s="251" t="s">
+        <v>246</v>
+      </c>
+      <c r="C13" s="240">
+        <v>768125</v>
+      </c>
+      <c r="D13" s="240">
+        <v>736664</v>
+      </c>
+      <c r="E13" s="252">
+        <f t="shared" si="0"/>
+        <v>31461</v>
+      </c>
+      <c r="H13" s="242"/>
+      <c r="I13" s="242"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="284" t="s">
+        <v>164</v>
+      </c>
+      <c r="B14" s="251" t="s">
+        <v>233</v>
+      </c>
+      <c r="C14" s="240">
+        <v>129240</v>
+      </c>
+      <c r="D14" s="240">
+        <v>120858</v>
+      </c>
+      <c r="E14" s="252">
+        <f t="shared" si="0"/>
+        <v>8382</v>
+      </c>
+      <c r="H14" s="241" t="s">
+        <v>241</v>
+      </c>
+      <c r="I14" s="243">
+        <v>4222963</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="284"/>
+      <c r="B15" s="251" t="s">
+        <v>234</v>
+      </c>
+      <c r="C15" s="240">
+        <v>133412</v>
+      </c>
+      <c r="D15" s="240">
+        <v>131583</v>
+      </c>
+      <c r="E15" s="252">
+        <f t="shared" si="0"/>
+        <v>1829</v>
+      </c>
+      <c r="H15" s="241" t="s">
+        <v>242</v>
+      </c>
+      <c r="I15" s="243">
+        <v>261494</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="284"/>
+      <c r="B16" s="251" t="s">
+        <v>235</v>
+      </c>
+      <c r="C16" s="240">
+        <v>152560</v>
+      </c>
+      <c r="D16" s="240">
+        <v>150810</v>
+      </c>
+      <c r="E16" s="252">
+        <f t="shared" si="0"/>
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="284"/>
+      <c r="B17" s="251" t="s">
+        <v>165</v>
+      </c>
+      <c r="C17" s="240">
+        <v>133725</v>
+      </c>
+      <c r="D17" s="240">
+        <v>133684</v>
+      </c>
+      <c r="E17" s="252">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="284"/>
+      <c r="B18" s="251" t="s">
+        <v>162</v>
+      </c>
+      <c r="C18" s="240">
+        <v>139600</v>
+      </c>
+      <c r="D18" s="240">
+        <v>136960</v>
+      </c>
+      <c r="E18" s="252">
+        <f t="shared" si="0"/>
+        <v>2640</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="284"/>
+      <c r="B19" s="251" t="s">
+        <v>163</v>
+      </c>
+      <c r="C19" s="240">
+        <v>146080</v>
+      </c>
+      <c r="D19" s="240">
+        <v>145437</v>
+      </c>
+      <c r="E19" s="252">
+        <f t="shared" si="0"/>
+        <v>643</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="284"/>
+      <c r="B20" s="251" t="s">
+        <v>246</v>
+      </c>
+      <c r="C20" s="240">
+        <v>219190</v>
+      </c>
+      <c r="D20" s="240">
+        <v>219190</v>
+      </c>
+      <c r="E20" s="252">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="284" t="s">
+        <v>166</v>
+      </c>
+      <c r="B21" s="251" t="s">
+        <v>233</v>
+      </c>
+      <c r="C21" s="240">
+        <v>0</v>
+      </c>
+      <c r="D21" s="240">
+        <v>0</v>
+      </c>
+      <c r="E21" s="252">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="284"/>
+      <c r="B22" s="251" t="s">
+        <v>234</v>
+      </c>
+      <c r="C22" s="240">
+        <v>109100</v>
+      </c>
+      <c r="D22" s="240">
+        <v>101841</v>
+      </c>
+      <c r="E22" s="252">
+        <f t="shared" si="0"/>
+        <v>7259</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="284"/>
+      <c r="B23" s="251" t="s">
+        <v>235</v>
+      </c>
+      <c r="C23" s="240">
+        <v>125510</v>
+      </c>
+      <c r="D23" s="240">
+        <v>103404</v>
+      </c>
+      <c r="E23" s="252">
+        <f t="shared" si="0"/>
+        <v>22106</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="284"/>
+      <c r="B24" s="251" t="s">
+        <v>165</v>
+      </c>
+      <c r="C24" s="240">
+        <v>108395</v>
+      </c>
+      <c r="D24" s="240">
+        <v>94818</v>
+      </c>
+      <c r="E24" s="252">
+        <f t="shared" si="0"/>
+        <v>13577</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="284"/>
+      <c r="B25" s="251" t="s">
+        <v>162</v>
+      </c>
+      <c r="C25" s="240">
+        <v>114100</v>
+      </c>
+      <c r="D25" s="240">
+        <v>104314</v>
+      </c>
+      <c r="E25" s="252">
+        <f t="shared" si="0"/>
+        <v>9786</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="284"/>
+      <c r="B26" s="251" t="s">
+        <v>163</v>
+      </c>
+      <c r="C26" s="240">
+        <v>119805</v>
+      </c>
+      <c r="D26" s="240">
+        <v>110598</v>
+      </c>
+      <c r="E26" s="252">
+        <f t="shared" si="0"/>
+        <v>9207</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="284"/>
+      <c r="B27" s="251" t="s">
+        <v>246</v>
+      </c>
+      <c r="C27" s="240">
+        <v>124775</v>
+      </c>
+      <c r="D27" s="240">
+        <v>124124</v>
+      </c>
+      <c r="E27" s="252">
+        <f t="shared" si="0"/>
+        <v>651</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="251" t="s">
+        <v>247</v>
+      </c>
+      <c r="B28" s="251" t="s">
+        <v>246</v>
+      </c>
+      <c r="C28" s="240">
+        <v>9800</v>
+      </c>
+      <c r="D28" s="240">
+        <v>9604</v>
+      </c>
+      <c r="E28" s="252">
+        <f t="shared" si="0"/>
+        <v>196</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="31" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="246" t="s">
+        <v>159</v>
+      </c>
+      <c r="B31" s="247" t="s">
+        <v>160</v>
+      </c>
+      <c r="C31" s="248" t="s">
+        <v>236</v>
+      </c>
+      <c r="D31" s="248" t="s">
+        <v>237</v>
+      </c>
+      <c r="E31" s="249" t="s">
+        <v>238</v>
+      </c>
+      <c r="F31" s="250" t="s">
+        <v>239</v>
+      </c>
+      <c r="G31" s="244"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="284" t="s">
+        <v>161</v>
+      </c>
+      <c r="B32" s="251" t="s">
+        <v>233</v>
+      </c>
+      <c r="C32" s="240">
+        <v>484110</v>
+      </c>
+      <c r="D32" s="240">
+        <v>484033</v>
+      </c>
+      <c r="E32" s="252">
+        <f t="shared" ref="E32:E53" si="1">C32-D32</f>
+        <v>77</v>
+      </c>
+      <c r="F32" s="253">
+        <f>E32/C32</f>
+        <v>1.5905476028175414E-4</v>
+      </c>
+      <c r="G32" s="283"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="284"/>
+      <c r="B33" s="251" t="s">
+        <v>234</v>
+      </c>
+      <c r="C33" s="240">
+        <v>442800</v>
+      </c>
+      <c r="D33" s="240">
+        <v>426896</v>
+      </c>
+      <c r="E33" s="252">
+        <f t="shared" si="1"/>
+        <v>15904</v>
+      </c>
+      <c r="F33" s="253">
+        <f t="shared" ref="F33:F53" si="2">E33/C33</f>
+        <v>3.5916892502258359E-2</v>
+      </c>
+      <c r="G33" s="283"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="284"/>
+      <c r="B34" s="251" t="s">
+        <v>235</v>
+      </c>
+      <c r="C34" s="240">
+        <v>513380</v>
+      </c>
+      <c r="D34" s="240">
+        <v>486936</v>
+      </c>
+      <c r="E34" s="252">
+        <f t="shared" si="1"/>
+        <v>26444</v>
+      </c>
+      <c r="F34" s="253">
+        <f t="shared" si="2"/>
+        <v>5.1509603023101799E-2</v>
+      </c>
+      <c r="G34" s="283"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="284"/>
+      <c r="B35" s="251" t="s">
+        <v>165</v>
+      </c>
+      <c r="C35" s="240">
+        <v>490800</v>
+      </c>
+      <c r="D35" s="240">
+        <v>441840</v>
+      </c>
+      <c r="E35" s="252">
+        <f t="shared" si="1"/>
+        <v>48960</v>
+      </c>
+      <c r="F35" s="253">
+        <f t="shared" si="2"/>
+        <v>9.9755501222493881E-2</v>
+      </c>
+      <c r="G35" s="283"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="284"/>
+      <c r="B36" s="251" t="s">
+        <v>162</v>
+      </c>
+      <c r="C36" s="240">
+        <v>524800</v>
+      </c>
+      <c r="D36" s="240">
+        <v>484326</v>
+      </c>
+      <c r="E36" s="252">
+        <f t="shared" si="1"/>
+        <v>40474</v>
+      </c>
+      <c r="F36" s="253">
+        <f t="shared" si="2"/>
+        <v>7.7122713414634142E-2</v>
+      </c>
+      <c r="G36" s="283"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="284"/>
+      <c r="B37" s="251" t="s">
+        <v>163</v>
+      </c>
+      <c r="C37" s="240">
+        <v>617040</v>
+      </c>
+      <c r="D37" s="240">
+        <v>564625</v>
+      </c>
+      <c r="E37" s="252">
         <f t="shared" si="1"/>
         <v>52415</v>
       </c>
-      <c r="H12" s="288" t="s">
-        <v>243</v>
-      </c>
-      <c r="I12" s="288" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="281" t="s">
+      <c r="F37" s="253">
+        <f t="shared" si="2"/>
+        <v>8.4945870608064314E-2</v>
+      </c>
+      <c r="G37" s="283"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="284"/>
+      <c r="B38" s="251" t="s">
+        <v>246</v>
+      </c>
+      <c r="C38" s="240">
+        <v>768125</v>
+      </c>
+      <c r="D38" s="240">
+        <v>736664</v>
+      </c>
+      <c r="E38" s="252">
+        <f t="shared" si="1"/>
+        <v>31461</v>
+      </c>
+      <c r="F38" s="253">
+        <f t="shared" si="2"/>
+        <v>4.0958177379983723E-2</v>
+      </c>
+      <c r="G38" s="245"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="284" t="s">
         <v>164</v>
       </c>
-      <c r="B13" s="241" t="s">
+      <c r="B39" s="251" t="s">
         <v>233</v>
       </c>
-      <c r="C13" s="247">
+      <c r="C39" s="240">
         <v>129240</v>
       </c>
-      <c r="D13" s="247">
+      <c r="D39" s="240">
         <v>120858</v>
       </c>
-      <c r="E13" s="248">
+      <c r="E39" s="252">
         <f t="shared" si="1"/>
         <v>8382</v>
       </c>
-      <c r="H13" s="287" t="s">
-        <v>241</v>
-      </c>
-      <c r="I13" s="289">
-        <v>4222963</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="282"/>
-      <c r="B14" s="239" t="s">
+      <c r="F39" s="253">
+        <f t="shared" si="2"/>
+        <v>6.4856081708449392E-2</v>
+      </c>
+      <c r="G39" s="283"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="284"/>
+      <c r="B40" s="251" t="s">
         <v>234</v>
       </c>
-      <c r="C14" s="249">
+      <c r="C40" s="240">
         <v>133412</v>
       </c>
-      <c r="D14" s="249">
+      <c r="D40" s="240">
         <v>131583</v>
       </c>
-      <c r="E14" s="248">
+      <c r="E40" s="252">
         <f t="shared" si="1"/>
         <v>1829</v>
       </c>
-      <c r="H14" s="287" t="s">
-        <v>242</v>
-      </c>
-      <c r="I14" s="289">
-        <v>261494</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="282"/>
-      <c r="B15" s="239" t="s">
+      <c r="F40" s="253">
+        <f t="shared" si="2"/>
+        <v>1.3709411447246125E-2</v>
+      </c>
+      <c r="G40" s="283"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="284"/>
+      <c r="B41" s="251" t="s">
         <v>235</v>
       </c>
-      <c r="C15" s="249">
+      <c r="C41" s="240">
         <v>152560</v>
       </c>
-      <c r="D15" s="249">
+      <c r="D41" s="240">
         <v>150810</v>
       </c>
-      <c r="E15" s="248">
+      <c r="E41" s="252">
         <f t="shared" si="1"/>
         <v>1750</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="282"/>
-      <c r="B16" s="239" t="s">
+      <c r="F41" s="253">
+        <f t="shared" si="2"/>
+        <v>1.1470896696381752E-2</v>
+      </c>
+      <c r="G41" s="283"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="284"/>
+      <c r="B42" s="251" t="s">
         <v>165</v>
       </c>
-      <c r="C16" s="249">
+      <c r="C42" s="240">
         <v>133725</v>
       </c>
-      <c r="D16" s="249">
+      <c r="D42" s="240">
         <v>133684</v>
       </c>
-      <c r="E16" s="248">
+      <c r="E42" s="252">
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="282"/>
-      <c r="B17" s="239" t="s">
+      <c r="F42" s="253">
+        <f t="shared" si="2"/>
+        <v>3.0659936436717143E-4</v>
+      </c>
+      <c r="G42" s="283"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="284"/>
+      <c r="B43" s="251" t="s">
         <v>162</v>
       </c>
-      <c r="C17" s="249">
+      <c r="C43" s="240">
         <v>139600</v>
       </c>
-      <c r="D17" s="249">
+      <c r="D43" s="240">
         <v>136960</v>
       </c>
-      <c r="E17" s="248">
+      <c r="E43" s="252">
         <f t="shared" si="1"/>
         <v>2640</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="283"/>
-      <c r="B18" s="242" t="s">
+      <c r="F43" s="253">
+        <f t="shared" si="2"/>
+        <v>1.8911174785100286E-2</v>
+      </c>
+      <c r="G43" s="283"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="284"/>
+      <c r="B44" s="251" t="s">
         <v>163</v>
       </c>
-      <c r="C18" s="250">
+      <c r="C44" s="240">
         <v>146080</v>
       </c>
-      <c r="D18" s="250">
+      <c r="D44" s="240">
         <v>145437</v>
       </c>
-      <c r="E18" s="251">
+      <c r="E44" s="252">
         <f t="shared" si="1"/>
         <v>643</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="281" t="s">
-        <v>166</v>
-      </c>
-      <c r="B19" s="241" t="s">
-        <v>233</v>
-      </c>
-      <c r="C19" s="247">
-        <v>0</v>
-      </c>
-      <c r="D19" s="247">
-        <v>0</v>
-      </c>
-      <c r="E19" s="248">
+      <c r="F44" s="253">
+        <f t="shared" si="2"/>
+        <v>4.4016976998904707E-3</v>
+      </c>
+      <c r="G44" s="283"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="284"/>
+      <c r="B45" s="251" t="s">
+        <v>246</v>
+      </c>
+      <c r="C45" s="240">
+        <v>219190</v>
+      </c>
+      <c r="D45" s="240">
+        <v>219190</v>
+      </c>
+      <c r="E45" s="252">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="282"/>
-      <c r="B20" s="239" t="s">
+      <c r="F45" s="253">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G45" s="245"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="284" t="s">
+        <v>166</v>
+      </c>
+      <c r="B46" s="251" t="s">
+        <v>233</v>
+      </c>
+      <c r="C46" s="240">
+        <v>0</v>
+      </c>
+      <c r="D46" s="240">
+        <v>0</v>
+      </c>
+      <c r="E46" s="252">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F46" s="253">
+        <v>0</v>
+      </c>
+      <c r="G46" s="283"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="284"/>
+      <c r="B47" s="251" t="s">
         <v>234</v>
       </c>
-      <c r="C20" s="249">
+      <c r="C47" s="240">
         <v>109100</v>
       </c>
-      <c r="D20" s="249">
+      <c r="D47" s="240">
         <v>101841</v>
       </c>
-      <c r="E20" s="248">
+      <c r="E47" s="252">
         <f t="shared" si="1"/>
         <v>7259</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="282"/>
-      <c r="B21" s="239" t="s">
+      <c r="F47" s="253">
+        <f t="shared" si="2"/>
+        <v>6.6535288725939501E-2</v>
+      </c>
+      <c r="G47" s="283"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="284"/>
+      <c r="B48" s="251" t="s">
         <v>235</v>
       </c>
-      <c r="C21" s="249">
+      <c r="C48" s="240">
         <v>125510</v>
       </c>
-      <c r="D21" s="249">
+      <c r="D48" s="240">
         <v>103404</v>
       </c>
-      <c r="E21" s="248">
+      <c r="E48" s="252">
         <f t="shared" si="1"/>
         <v>22106</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="282"/>
-      <c r="B22" s="239" t="s">
+      <c r="F48" s="253">
+        <f t="shared" si="2"/>
+        <v>0.17612939208031234</v>
+      </c>
+      <c r="G48" s="283"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="284"/>
+      <c r="B49" s="251" t="s">
         <v>165</v>
       </c>
-      <c r="C22" s="249">
+      <c r="C49" s="240">
         <v>108395</v>
       </c>
-      <c r="D22" s="249">
+      <c r="D49" s="240">
         <v>94818</v>
       </c>
-      <c r="E22" s="248">
+      <c r="E49" s="252">
         <f t="shared" si="1"/>
         <v>13577</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="282"/>
-      <c r="B23" s="239" t="s">
+      <c r="F49" s="253">
+        <f t="shared" si="2"/>
+        <v>0.12525485492873287</v>
+      </c>
+      <c r="G49" s="283"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="284"/>
+      <c r="B50" s="251" t="s">
         <v>162</v>
       </c>
-      <c r="C23" s="249">
+      <c r="C50" s="240">
         <v>114100</v>
       </c>
-      <c r="D23" s="249">
+      <c r="D50" s="240">
         <v>104314</v>
       </c>
-      <c r="E23" s="248">
+      <c r="E50" s="252">
         <f t="shared" si="1"/>
         <v>9786</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="283"/>
-      <c r="B24" s="242" t="s">
+      <c r="F50" s="253">
+        <f t="shared" si="2"/>
+        <v>8.5766871165644173E-2</v>
+      </c>
+      <c r="G50" s="283"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="284"/>
+      <c r="B51" s="251" t="s">
         <v>163</v>
       </c>
-      <c r="C24" s="250">
+      <c r="C51" s="240">
         <v>119805</v>
       </c>
-      <c r="D24" s="250">
+      <c r="D51" s="240">
         <v>110598</v>
       </c>
-      <c r="E24" s="251">
+      <c r="E51" s="252">
         <f t="shared" si="1"/>
         <v>9207</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="1:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="243" t="s">
-        <v>159</v>
-      </c>
-      <c r="B27" s="244" t="s">
-        <v>160</v>
-      </c>
-      <c r="C27" s="245" t="s">
-        <v>236</v>
-      </c>
-      <c r="D27" s="245" t="s">
-        <v>237</v>
-      </c>
-      <c r="E27" s="284" t="s">
-        <v>238</v>
-      </c>
-      <c r="F27" s="292" t="s">
-        <v>239</v>
-      </c>
-      <c r="G27" s="290"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="281" t="s">
-        <v>161</v>
-      </c>
-      <c r="B28" s="241" t="s">
-        <v>233</v>
-      </c>
-      <c r="C28" s="247">
-        <v>484110</v>
-      </c>
-      <c r="D28" s="247">
-        <f>390370+93663</f>
-        <v>484033</v>
-      </c>
-      <c r="E28" s="285">
-        <f t="shared" ref="E28:E30" si="2">C28-D28</f>
-        <v>77</v>
-      </c>
-      <c r="F28" s="293">
-        <f>E28/C28</f>
-        <v>1.5905476028175414E-4</v>
-      </c>
-      <c r="G28" s="291"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="282"/>
-      <c r="B29" s="252" t="s">
-        <v>234</v>
-      </c>
-      <c r="C29" s="249">
-        <v>442800</v>
-      </c>
-      <c r="D29" s="249">
-        <v>426896</v>
-      </c>
-      <c r="E29" s="285">
+      <c r="F51" s="253">
         <f t="shared" si="2"/>
-        <v>15904</v>
-      </c>
-      <c r="F29" s="293">
-        <f t="shared" ref="F29:F45" si="3">E29/C29</f>
-        <v>3.5916892502258359E-2</v>
-      </c>
-      <c r="G29" s="291"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="282"/>
-      <c r="B30" s="252" t="s">
-        <v>235</v>
-      </c>
-      <c r="C30" s="249">
-        <v>513380</v>
-      </c>
-      <c r="D30" s="249">
-        <v>486936</v>
-      </c>
-      <c r="E30" s="285">
+        <v>7.6849881056717168E-2</v>
+      </c>
+      <c r="G51" s="283"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="284"/>
+      <c r="B52" s="251" t="s">
+        <v>246</v>
+      </c>
+      <c r="C52" s="240">
+        <v>124775</v>
+      </c>
+      <c r="D52" s="240">
+        <v>124124</v>
+      </c>
+      <c r="E52" s="252">
+        <f t="shared" si="1"/>
+        <v>651</v>
+      </c>
+      <c r="F52" s="253">
         <f t="shared" si="2"/>
-        <v>26444</v>
-      </c>
-      <c r="F30" s="293">
-        <f t="shared" si="3"/>
-        <v>5.1509603023101799E-2</v>
-      </c>
-      <c r="G30" s="291"/>
-    </row>
-    <row r="31" spans="1:7" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="282"/>
-      <c r="B31" s="252" t="s">
-        <v>165</v>
-      </c>
-      <c r="C31" s="249">
-        <v>490800</v>
-      </c>
-      <c r="D31" s="249">
-        <v>441840</v>
-      </c>
-      <c r="E31" s="285">
-        <f>C31-D31</f>
-        <v>48960</v>
-      </c>
-      <c r="F31" s="293">
-        <f t="shared" si="3"/>
-        <v>9.9755501222493881E-2</v>
-      </c>
-      <c r="G31" s="291"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="282"/>
-      <c r="B32" s="252" t="s">
-        <v>162</v>
-      </c>
-      <c r="C32" s="249">
-        <v>524800</v>
-      </c>
-      <c r="D32" s="249">
-        <v>484326</v>
-      </c>
-      <c r="E32" s="285">
-        <f t="shared" ref="E32:E45" si="4">C32-D32</f>
-        <v>40474</v>
-      </c>
-      <c r="F32" s="293">
-        <f t="shared" si="3"/>
-        <v>7.7122713414634142E-2</v>
-      </c>
-      <c r="G32" s="291"/>
-    </row>
-    <row r="33" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="283"/>
-      <c r="B33" s="242" t="s">
-        <v>163</v>
-      </c>
-      <c r="C33" s="250">
-        <v>617040</v>
-      </c>
-      <c r="D33" s="250">
-        <v>564625</v>
-      </c>
-      <c r="E33" s="286">
-        <f t="shared" si="4"/>
-        <v>52415</v>
-      </c>
-      <c r="F33" s="293">
-        <f t="shared" si="3"/>
-        <v>8.4945870608064314E-2</v>
-      </c>
-      <c r="G33" s="291"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="281" t="s">
-        <v>164</v>
-      </c>
-      <c r="B34" s="241" t="s">
-        <v>233</v>
-      </c>
-      <c r="C34" s="247">
-        <v>129240</v>
-      </c>
-      <c r="D34" s="247">
-        <v>120858</v>
-      </c>
-      <c r="E34" s="285">
-        <f t="shared" si="4"/>
-        <v>8382</v>
-      </c>
-      <c r="F34" s="293">
-        <f t="shared" si="3"/>
-        <v>6.4856081708449392E-2</v>
-      </c>
-      <c r="G34" s="291"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="282"/>
-      <c r="B35" s="252" t="s">
-        <v>234</v>
-      </c>
-      <c r="C35" s="249">
-        <v>133412</v>
-      </c>
-      <c r="D35" s="249">
-        <v>131583</v>
-      </c>
-      <c r="E35" s="285">
-        <f t="shared" si="4"/>
-        <v>1829</v>
-      </c>
-      <c r="F35" s="293">
-        <f t="shared" si="3"/>
-        <v>1.3709411447246125E-2</v>
-      </c>
-      <c r="G35" s="291"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="282"/>
-      <c r="B36" s="252" t="s">
-        <v>235</v>
-      </c>
-      <c r="C36" s="249">
-        <v>152560</v>
-      </c>
-      <c r="D36" s="249">
-        <v>150810</v>
-      </c>
-      <c r="E36" s="285">
-        <f t="shared" si="4"/>
-        <v>1750</v>
-      </c>
-      <c r="F36" s="293">
-        <f t="shared" si="3"/>
-        <v>1.1470896696381752E-2</v>
-      </c>
-      <c r="G36" s="291"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="282"/>
-      <c r="B37" s="252" t="s">
-        <v>165</v>
-      </c>
-      <c r="C37" s="249">
-        <v>133725</v>
-      </c>
-      <c r="D37" s="249">
-        <v>133684</v>
-      </c>
-      <c r="E37" s="285">
-        <f t="shared" si="4"/>
-        <v>41</v>
-      </c>
-      <c r="F37" s="293">
-        <f t="shared" si="3"/>
-        <v>3.0659936436717143E-4</v>
-      </c>
-      <c r="G37" s="291"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="282"/>
-      <c r="B38" s="252" t="s">
-        <v>162</v>
-      </c>
-      <c r="C38" s="249">
-        <v>139600</v>
-      </c>
-      <c r="D38" s="249">
-        <v>136960</v>
-      </c>
-      <c r="E38" s="285">
-        <f t="shared" si="4"/>
-        <v>2640</v>
-      </c>
-      <c r="F38" s="293">
-        <f t="shared" si="3"/>
-        <v>1.8911174785100286E-2</v>
-      </c>
-      <c r="G38" s="291"/>
-    </row>
-    <row r="39" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="283"/>
-      <c r="B39" s="242" t="s">
-        <v>163</v>
-      </c>
-      <c r="C39" s="250">
-        <v>146080</v>
-      </c>
-      <c r="D39" s="250">
-        <v>145437</v>
-      </c>
-      <c r="E39" s="286">
-        <f t="shared" si="4"/>
-        <v>643</v>
-      </c>
-      <c r="F39" s="293">
-        <f t="shared" si="3"/>
-        <v>4.4016976998904707E-3</v>
-      </c>
-      <c r="G39" s="291"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="281" t="s">
-        <v>166</v>
-      </c>
-      <c r="B40" s="241" t="s">
-        <v>233</v>
-      </c>
-      <c r="C40" s="247">
-        <v>0</v>
-      </c>
-      <c r="D40" s="247">
-        <v>0</v>
-      </c>
-      <c r="E40" s="285">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="F40" s="293">
-        <v>0</v>
-      </c>
-      <c r="G40" s="291"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="282"/>
-      <c r="B41" s="252" t="s">
-        <v>234</v>
-      </c>
-      <c r="C41" s="249">
-        <v>109100</v>
-      </c>
-      <c r="D41" s="249">
-        <v>101841</v>
-      </c>
-      <c r="E41" s="285">
-        <f t="shared" si="4"/>
-        <v>7259</v>
-      </c>
-      <c r="F41" s="293">
-        <f t="shared" si="3"/>
-        <v>6.6535288725939501E-2</v>
-      </c>
-      <c r="G41" s="291"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="282"/>
-      <c r="B42" s="252" t="s">
-        <v>235</v>
-      </c>
-      <c r="C42" s="249">
-        <v>125510</v>
-      </c>
-      <c r="D42" s="249">
-        <v>103404</v>
-      </c>
-      <c r="E42" s="285">
-        <f t="shared" si="4"/>
-        <v>22106</v>
-      </c>
-      <c r="F42" s="293">
-        <f t="shared" si="3"/>
-        <v>0.17612939208031234</v>
-      </c>
-      <c r="G42" s="291"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" s="282"/>
-      <c r="B43" s="252" t="s">
-        <v>165</v>
-      </c>
-      <c r="C43" s="249">
-        <v>108395</v>
-      </c>
-      <c r="D43" s="249">
-        <v>94818</v>
-      </c>
-      <c r="E43" s="285">
-        <f t="shared" si="4"/>
-        <v>13577</v>
-      </c>
-      <c r="F43" s="293">
-        <f t="shared" si="3"/>
-        <v>0.12525485492873287</v>
-      </c>
-      <c r="G43" s="291"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="282"/>
-      <c r="B44" s="252" t="s">
-        <v>162</v>
-      </c>
-      <c r="C44" s="249">
-        <v>114100</v>
-      </c>
-      <c r="D44" s="249">
-        <v>104314</v>
-      </c>
-      <c r="E44" s="285">
-        <f t="shared" si="4"/>
-        <v>9786</v>
-      </c>
-      <c r="F44" s="293">
-        <f t="shared" si="3"/>
-        <v>8.5766871165644173E-2</v>
-      </c>
-      <c r="G44" s="291"/>
-    </row>
-    <row r="45" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="283"/>
-      <c r="B45" s="242" t="s">
-        <v>163</v>
-      </c>
-      <c r="C45" s="250">
-        <v>119805</v>
-      </c>
-      <c r="D45" s="250">
-        <v>110598</v>
-      </c>
-      <c r="E45" s="286">
-        <f t="shared" si="4"/>
-        <v>9207</v>
-      </c>
-      <c r="F45" s="294">
-        <f t="shared" si="3"/>
-        <v>7.6849881056717168E-2</v>
-      </c>
-      <c r="G45" s="291"/>
-    </row>
-    <row r="51" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F51" s="240"/>
-    </row>
-    <row r="52" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F52" s="240"/>
-    </row>
-    <row r="53" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F53" s="240"/>
-    </row>
-    <row r="54" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F54" s="240"/>
-    </row>
-    <row r="55" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F55" s="240"/>
-    </row>
-    <row r="56" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F56" s="240"/>
-    </row>
-    <row r="57" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F57" s="240"/>
-    </row>
-    <row r="58" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F58" s="240"/>
-    </row>
-    <row r="59" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C59"/>
-      <c r="F59" s="240"/>
-    </row>
-    <row r="60" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C60"/>
-      <c r="F60" s="240"/>
-    </row>
-    <row r="61" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C61"/>
-      <c r="F61" s="240"/>
-    </row>
-    <row r="62" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C62"/>
-      <c r="F62" s="240"/>
-    </row>
-    <row r="63" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F63" s="240"/>
-    </row>
-    <row r="64" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F64" s="240"/>
-    </row>
-    <row r="65" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F65" s="240"/>
-    </row>
-    <row r="66" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F66" s="240"/>
-    </row>
-    <row r="67" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F67" s="240"/>
-    </row>
-    <row r="68" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F68" s="240"/>
-    </row>
-    <row r="69" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F69" s="240"/>
+        <v>5.2173913043478265E-3</v>
+      </c>
+      <c r="G52" s="245"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="251" t="s">
+        <v>247</v>
+      </c>
+      <c r="B53" s="251" t="s">
+        <v>246</v>
+      </c>
+      <c r="C53" s="240">
+        <v>9800</v>
+      </c>
+      <c r="D53" s="240">
+        <v>9604</v>
+      </c>
+      <c r="E53" s="252">
+        <f t="shared" si="1"/>
+        <v>196</v>
+      </c>
+      <c r="F53" s="253">
+        <f t="shared" si="2"/>
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F58" s="239"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F59" s="239"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F60" s="239"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F61" s="239"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F62" s="239"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F63" s="239"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F64" s="239"/>
+    </row>
+    <row r="65" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="F65" s="239"/>
+    </row>
+    <row r="66" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C66"/>
+      <c r="F66" s="239"/>
+    </row>
+    <row r="67" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C67"/>
+      <c r="F67" s="239"/>
+    </row>
+    <row r="68" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C68"/>
+      <c r="F68" s="239"/>
+    </row>
+    <row r="69" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C69"/>
+      <c r="F69" s="239"/>
+    </row>
+    <row r="70" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="F70" s="239"/>
+    </row>
+    <row r="71" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="F71" s="239"/>
+    </row>
+    <row r="72" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="F72" s="239"/>
+    </row>
+    <row r="73" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="F73" s="239"/>
+    </row>
+    <row r="74" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="F74" s="239"/>
+    </row>
+    <row r="75" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="F75" s="239"/>
+    </row>
+    <row r="76" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="F76" s="239"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="G28:G33"/>
-    <mergeCell ref="G34:G39"/>
-    <mergeCell ref="G40:G45"/>
-    <mergeCell ref="A7:A12"/>
-    <mergeCell ref="A13:A18"/>
-    <mergeCell ref="A19:A24"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="A34:A39"/>
-    <mergeCell ref="A40:A45"/>
+    <mergeCell ref="G46:G51"/>
+    <mergeCell ref="A39:A45"/>
+    <mergeCell ref="A32:A38"/>
+    <mergeCell ref="A46:A52"/>
+    <mergeCell ref="A7:A13"/>
+    <mergeCell ref="A14:A20"/>
+    <mergeCell ref="A21:A27"/>
+    <mergeCell ref="G32:G37"/>
+    <mergeCell ref="G39:G44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -70083,7 +70125,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>

</xml_diff>